<commit_message>
Add Sonny Moore as 4th ensemble system — RMSE drops to 3.2%
4-system ensemble: Torvik (35%) + SR Adjusted (25%) + ESPN BPI (25%) +
Sonny Moore (15%). Average deviation from Vegas: 3.2 percentage points.

Progression: 5.7% → 4.1% → 3.7% → 3.6% → 3.2%

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/march_madness_2026_brackets.xlsx
+++ b/output/march_madness_2026_brackets.xlsx
@@ -870,19 +870,19 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0.98728</v>
+        <v>0.9886</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.85802</v>
+        <v>0.8641</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.68168</v>
+        <v>0.68834</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>0.50584</v>
+        <v>0.5162600000000001</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.20802</v>
+        <v>0.21246</v>
       </c>
     </row>
     <row r="5">
@@ -900,19 +900,19 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.99216</v>
+        <v>0.99296</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.8502</v>
+        <v>0.86032</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.66292</v>
+        <v>0.6768999999999999</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.45502</v>
+        <v>0.465</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.15586</v>
+        <v>0.15978</v>
       </c>
     </row>
     <row r="6">
@@ -930,19 +930,19 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>0.99124</v>
+        <v>0.992</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.83492</v>
+        <v>0.84306</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.6324</v>
+        <v>0.64122</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.43286</v>
+        <v>0.4417</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.14568</v>
+        <v>0.14904</v>
       </c>
     </row>
     <row r="7">
@@ -960,19 +960,19 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0.99466</v>
+        <v>0.99524</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.81494</v>
+        <v>0.82194</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.58966</v>
+        <v>0.59838</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.33448</v>
+        <v>0.34072</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.09528</v>
+        <v>0.09637999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -990,19 +990,19 @@
         </is>
       </c>
       <c r="D8" s="9" t="n">
-        <v>0.96836</v>
+        <v>0.97112</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.76528</v>
+        <v>0.78012</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0.47212</v>
+        <v>0.4789</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.27652</v>
+        <v>0.27826</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>0.07876</v>
+        <v>0.07716000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -1020,19 +1020,19 @@
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.9719</v>
+        <v>0.97356</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.7627</v>
+        <v>0.77188</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>0.48796</v>
+        <v>0.4946</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>0.2417</v>
+        <v>0.24276</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>0.05528</v>
+        <v>0.0547</v>
       </c>
     </row>
     <row r="10">
@@ -1050,19 +1050,19 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>0.9723000000000001</v>
+        <v>0.97406</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0.77438</v>
+        <v>0.79028</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.50754</v>
+        <v>0.5226</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.24582</v>
+        <v>0.24966</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>0.0517</v>
+        <v>0.05176</v>
       </c>
     </row>
     <row r="11">
@@ -1080,19 +1080,19 @@
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>0.95272</v>
+        <v>0.95524</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>0.78988</v>
+        <v>0.79436</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.40818</v>
+        <v>0.4116</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>0.21866</v>
+        <v>0.21932</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>0.05154</v>
+        <v>0.05102</v>
       </c>
     </row>
     <row r="12">
@@ -1110,19 +1110,19 @@
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>0.96228</v>
+        <v>0.96432</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>0.71354</v>
+        <v>0.70966</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0.39986</v>
+        <v>0.38572</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.1572</v>
+        <v>0.1444</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>0.02944</v>
+        <v>0.02416</v>
       </c>
     </row>
     <row r="13">
@@ -1140,19 +1140,19 @@
         </is>
       </c>
       <c r="D13" s="9" t="n">
-        <v>0.9243400000000001</v>
+        <v>0.93308</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>0.5698800000000001</v>
+        <v>0.57808</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>0.31188</v>
+        <v>0.32622</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>0.11922</v>
+        <v>0.12334</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>0.02004</v>
+        <v>0.02046</v>
       </c>
     </row>
     <row r="14">
@@ -1170,19 +1170,19 @@
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>0.93326</v>
+        <v>0.9348</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>0.6916</v>
+        <v>0.69738</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.33262</v>
+        <v>0.33044</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.13284</v>
+        <v>0.12794</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>0.01842</v>
+        <v>0.01694</v>
       </c>
     </row>
     <row r="15">
@@ -1200,19 +1200,19 @@
         </is>
       </c>
       <c r="D15" s="13" t="n">
-        <v>0.90522</v>
+        <v>0.91082</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>0.5678800000000001</v>
+        <v>0.57486</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>0.19148</v>
+        <v>0.19122</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>0.08938</v>
+        <v>0.09034</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.01124</v>
+        <v>0.01136</v>
       </c>
     </row>
     <row r="16">
@@ -1230,19 +1230,19 @@
         </is>
       </c>
       <c r="D16" s="13" t="n">
-        <v>0.7423999999999999</v>
+        <v>0.75752</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.41768</v>
+        <v>0.41876</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>0.19516</v>
+        <v>0.19302</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>0.07528</v>
+        <v>0.073</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.01054</v>
+        <v>0.01012</v>
       </c>
     </row>
     <row r="17">
@@ -1260,79 +1260,79 @@
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>0.92132</v>
-      </c>
-      <c r="E17" s="10" t="n">
-        <v>0.49746</v>
+        <v>0.92496</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>0.50798</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>0.218</v>
+        <v>0.22338</v>
       </c>
       <c r="G17" s="10" t="n">
-        <v>0.07904</v>
+        <v>0.08037999999999999</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>0.0098</v>
+        <v>0.01004</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>St. John's</t>
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D18" s="13" t="n">
-        <v>0.87526</v>
+        <v>0.83602</v>
       </c>
       <c r="E18" s="13" t="n">
-        <v>0.56724</v>
+        <v>0.53416</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>0.18226</v>
+        <v>0.15902</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>0.07852000000000001</v>
+        <v>0.07858</v>
       </c>
       <c r="H18" s="14" t="n">
-        <v>0.00958</v>
+        <v>0.0098</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>St. John's</t>
+          <t>Alabama</t>
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="D19" s="13" t="n">
-        <v>0.83578</v>
+        <v>0.87356</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>0.52898</v>
+        <v>0.57312</v>
       </c>
       <c r="F19" s="14" t="n">
-        <v>0.15898</v>
+        <v>0.17932</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>0.07692</v>
+        <v>0.07622</v>
       </c>
       <c r="H19" s="14" t="n">
-        <v>0.009560000000000001</v>
+        <v>0.00894</v>
       </c>
     </row>
     <row r="20">
@@ -1350,19 +1350,19 @@
         </is>
       </c>
       <c r="D20" s="13" t="n">
-        <v>0.81504</v>
+        <v>0.81028</v>
       </c>
       <c r="E20" s="14" t="n">
-        <v>0.48274</v>
+        <v>0.48016</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>0.18352</v>
+        <v>0.18028</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>0.07031999999999999</v>
+        <v>0.06876</v>
       </c>
       <c r="H20" s="14" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.00838</v>
       </c>
     </row>
     <row r="21">
@@ -1380,19 +1380,19 @@
         </is>
       </c>
       <c r="D21" s="13" t="n">
-        <v>0.76752</v>
+        <v>0.7607</v>
       </c>
       <c r="E21" s="14" t="n">
-        <v>0.37016</v>
+        <v>0.36204</v>
       </c>
       <c r="F21" s="14" t="n">
-        <v>0.18106</v>
+        <v>0.18162</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>0.06018</v>
+        <v>0.05946</v>
       </c>
       <c r="H21" s="14" t="n">
-        <v>0.00766</v>
+        <v>0.00728</v>
       </c>
     </row>
     <row r="22">
@@ -1410,19 +1410,19 @@
         </is>
       </c>
       <c r="D22" s="13" t="n">
-        <v>0.90668</v>
+        <v>0.91266</v>
       </c>
       <c r="E22" s="14" t="n">
-        <v>0.46386</v>
+        <v>0.46592</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>0.15386</v>
+        <v>0.1513</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>0.05126</v>
+        <v>0.04986</v>
       </c>
       <c r="H22" s="14" t="n">
-        <v>0.00476</v>
+        <v>0.00444</v>
       </c>
     </row>
     <row r="23">
@@ -1440,19 +1440,19 @@
         </is>
       </c>
       <c r="D23" s="13" t="n">
-        <v>0.8137</v>
+        <v>0.81852</v>
       </c>
       <c r="E23" s="14" t="n">
-        <v>0.38616</v>
+        <v>0.38288</v>
       </c>
       <c r="F23" s="14" t="n">
-        <v>0.11074</v>
+        <v>0.10728</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>0.04476</v>
+        <v>0.04274</v>
       </c>
       <c r="H23" s="14" t="n">
-        <v>0.00416</v>
+        <v>0.00392</v>
       </c>
     </row>
     <row r="24">
@@ -1470,19 +1470,19 @@
         </is>
       </c>
       <c r="D24" s="13" t="n">
-        <v>0.87598</v>
+        <v>0.87954</v>
       </c>
       <c r="E24" s="14" t="n">
-        <v>0.41616</v>
+        <v>0.41178</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>0.09916</v>
+        <v>0.09551999999999999</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>0.03824</v>
+        <v>0.03728</v>
       </c>
       <c r="H24" s="14" t="n">
-        <v>0.00322</v>
+        <v>0.00288</v>
       </c>
     </row>
     <row r="25">
@@ -1500,25 +1500,25 @@
         </is>
       </c>
       <c r="D25" s="13" t="n">
-        <v>0.76544</v>
+        <v>0.75182</v>
       </c>
       <c r="E25" s="14" t="n">
-        <v>0.35592</v>
+        <v>0.34324</v>
       </c>
       <c r="F25" s="14" t="n">
-        <v>0.08978</v>
+        <v>0.08232</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>0.03228</v>
+        <v>0.02872</v>
       </c>
       <c r="H25" s="14" t="n">
-        <v>0.00224</v>
+        <v>0.00176</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>Saint Mary's</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="B26" s="16" t="n">
@@ -1526,29 +1526,29 @@
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D26" s="17" t="n">
-        <v>0.60248</v>
+        <v>0.73268</v>
       </c>
       <c r="E26" s="18" t="n">
-        <v>0.15344</v>
+        <v>0.24508</v>
       </c>
       <c r="F26" s="18" t="n">
-        <v>0.05384</v>
+        <v>0.08672000000000001</v>
       </c>
       <c r="G26" s="18" t="n">
-        <v>0.01718</v>
+        <v>0.02006</v>
       </c>
       <c r="H26" s="18" t="n">
-        <v>0.0013</v>
+        <v>0.00122</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Saint Mary's</t>
         </is>
       </c>
       <c r="B27" s="16" t="n">
@@ -1556,23 +1556,23 @@
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>South</t>
         </is>
       </c>
       <c r="D27" s="17" t="n">
-        <v>0.72096</v>
+        <v>0.58612</v>
       </c>
       <c r="E27" s="18" t="n">
-        <v>0.2371</v>
+        <v>0.13778</v>
       </c>
       <c r="F27" s="18" t="n">
-        <v>0.08654000000000001</v>
+        <v>0.04496</v>
       </c>
       <c r="G27" s="18" t="n">
-        <v>0.0208</v>
+        <v>0.01338</v>
       </c>
       <c r="H27" s="18" t="n">
-        <v>0.00126</v>
+        <v>0.00096</v>
       </c>
     </row>
     <row r="28">
@@ -1590,79 +1590,79 @@
         </is>
       </c>
       <c r="D28" s="17" t="n">
-        <v>0.60936</v>
+        <v>0.60728</v>
       </c>
       <c r="E28" s="18" t="n">
-        <v>0.0983</v>
+        <v>0.09426</v>
       </c>
       <c r="F28" s="18" t="n">
-        <v>0.04282</v>
+        <v>0.04048</v>
       </c>
       <c r="G28" s="18" t="n">
-        <v>0.015</v>
+        <v>0.01424</v>
       </c>
       <c r="H28" s="18" t="n">
-        <v>0.00078</v>
+        <v>0.00066</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>BYU</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="n">
+        <v>0.61468</v>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>0.2029</v>
+      </c>
+      <c r="F29" s="14" t="n">
+        <v>0.05728</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>0.01216</v>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>0.00062</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>Miami FL</t>
         </is>
       </c>
-      <c r="B29" s="16" t="n">
+      <c r="B30" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="D29" s="17" t="n">
-        <v>0.6402600000000001</v>
-      </c>
-      <c r="E29" s="18" t="n">
-        <v>0.16224</v>
-      </c>
-      <c r="F29" s="18" t="n">
-        <v>0.06396</v>
-      </c>
-      <c r="G29" s="18" t="n">
-        <v>0.0158</v>
-      </c>
-      <c r="H29" s="18" t="n">
-        <v>0.00072</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>BYU</t>
-        </is>
-      </c>
-      <c r="B30" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="n">
-        <v>0.59714</v>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>0.19814</v>
-      </c>
-      <c r="F30" s="14" t="n">
-        <v>0.05674</v>
-      </c>
-      <c r="G30" s="14" t="n">
-        <v>0.01246</v>
-      </c>
-      <c r="H30" s="14" t="n">
-        <v>0.0006400000000000001</v>
+      <c r="D30" s="17" t="n">
+        <v>0.61854</v>
+      </c>
+      <c r="E30" s="18" t="n">
+        <v>0.14376</v>
+      </c>
+      <c r="F30" s="18" t="n">
+        <v>0.0536</v>
+      </c>
+      <c r="G30" s="18" t="n">
+        <v>0.01204</v>
+      </c>
+      <c r="H30" s="18" t="n">
+        <v>0.00052</v>
       </c>
     </row>
     <row r="31">
@@ -1680,19 +1680,19 @@
         </is>
       </c>
       <c r="D31" s="17" t="n">
-        <v>0.53498</v>
+        <v>0.54042</v>
       </c>
       <c r="E31" s="18" t="n">
-        <v>0.09397999999999999</v>
+        <v>0.09136</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>0.03742</v>
+        <v>0.03556</v>
       </c>
       <c r="G31" s="18" t="n">
-        <v>0.0124</v>
+        <v>0.01168</v>
       </c>
       <c r="H31" s="18" t="n">
-        <v>0.00052</v>
+        <v>0.00048</v>
       </c>
     </row>
     <row r="32">
@@ -1710,139 +1710,139 @@
         </is>
       </c>
       <c r="D32" s="13" t="n">
-        <v>0.60532</v>
+        <v>0.5939</v>
       </c>
       <c r="E32" s="14" t="n">
-        <v>0.13878</v>
+        <v>0.1325</v>
       </c>
       <c r="F32" s="14" t="n">
-        <v>0.0318</v>
+        <v>0.03004</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>0.00762</v>
+        <v>0.007</v>
       </c>
       <c r="H32" s="14" t="n">
-        <v>0.00048</v>
+        <v>0.00042</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="B33" s="16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="D33" s="17" t="n">
-        <v>0.53712</v>
+        <v>0.54308</v>
       </c>
       <c r="E33" s="18" t="n">
-        <v>0.1062</v>
+        <v>0.08024000000000001</v>
       </c>
       <c r="F33" s="18" t="n">
-        <v>0.04036</v>
+        <v>0.0329</v>
       </c>
       <c r="G33" s="18" t="n">
-        <v>0.00974</v>
+        <v>0.00924</v>
       </c>
       <c r="H33" s="18" t="n">
-        <v>0.00044</v>
+        <v>0.00042</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="B34" s="16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>South</t>
         </is>
       </c>
       <c r="D34" s="17" t="n">
-        <v>0.5213</v>
+        <v>0.53738</v>
       </c>
       <c r="E34" s="18" t="n">
-        <v>0.07974000000000001</v>
+        <v>0.10242</v>
       </c>
       <c r="F34" s="18" t="n">
-        <v>0.03238</v>
+        <v>0.03854</v>
       </c>
       <c r="G34" s="18" t="n">
-        <v>0.00928</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="H34" s="18" t="n">
-        <v>0.00042</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Villanova</t>
         </is>
       </c>
       <c r="B35" s="16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>Midwest</t>
-        </is>
-      </c>
-      <c r="D35" s="17" t="n">
-        <v>0.54372</v>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="D35" s="18" t="n">
+        <v>0.45958</v>
       </c>
       <c r="E35" s="18" t="n">
-        <v>0.13294</v>
+        <v>0.06516</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>0.04756</v>
+        <v>0.02232</v>
       </c>
       <c r="G35" s="18" t="n">
-        <v>0.01122</v>
+        <v>0.00624</v>
       </c>
       <c r="H35" s="18" t="n">
-        <v>0.00034</v>
+        <v>0.00026</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>Villanova</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="B36" s="16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="D36" s="18" t="n">
-        <v>0.46502</v>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="n">
+        <v>0.5455</v>
       </c>
       <c r="E36" s="18" t="n">
-        <v>0.07054000000000001</v>
+        <v>0.12846</v>
       </c>
       <c r="F36" s="18" t="n">
-        <v>0.02514</v>
+        <v>0.0444</v>
       </c>
       <c r="G36" s="18" t="n">
-        <v>0.00722</v>
+        <v>0.01024</v>
       </c>
       <c r="H36" s="18" t="n">
-        <v>0.00032</v>
+        <v>0.00026</v>
       </c>
     </row>
     <row r="37">
@@ -1860,16 +1860,16 @@
         </is>
       </c>
       <c r="D37" s="18" t="n">
-        <v>0.46288</v>
+        <v>0.46262</v>
       </c>
       <c r="E37" s="18" t="n">
-        <v>0.07876</v>
+        <v>0.07557999999999999</v>
       </c>
       <c r="F37" s="18" t="n">
-        <v>0.02678</v>
+        <v>0.02532</v>
       </c>
       <c r="G37" s="18" t="n">
-        <v>0.00586</v>
+        <v>0.00542</v>
       </c>
       <c r="H37" s="18" t="n">
         <v>0.00024</v>
@@ -1878,7 +1878,7 @@
     <row r="38">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>Texas A&amp;M</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -1886,53 +1886,53 @@
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>South</t>
         </is>
       </c>
       <c r="D38" s="21" t="n">
-        <v>0.45628</v>
+        <v>0.41388</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>0.10238</v>
+        <v>0.0795</v>
       </c>
       <c r="F38" s="21" t="n">
-        <v>0.03332</v>
+        <v>0.02202</v>
       </c>
       <c r="G38" s="21" t="n">
-        <v>0.00738</v>
+        <v>0.0051</v>
       </c>
       <c r="H38" s="21" t="n">
-        <v>0.0002</v>
+        <v>0.00016</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>Texas A&amp;M</t>
-        </is>
-      </c>
-      <c r="B39" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="C39" s="19" t="inlineStr">
-        <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="D39" s="21" t="n">
-        <v>0.39752</v>
-      </c>
-      <c r="E39" s="21" t="n">
-        <v>0.07824</v>
-      </c>
-      <c r="F39" s="21" t="n">
-        <v>0.02242</v>
-      </c>
-      <c r="G39" s="21" t="n">
-        <v>0.00548</v>
-      </c>
-      <c r="H39" s="21" t="n">
-        <v>0.00018</v>
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>TCU</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D39" s="18" t="n">
+        <v>0.39272</v>
+      </c>
+      <c r="E39" s="18" t="n">
+        <v>0.0409</v>
+      </c>
+      <c r="F39" s="18" t="n">
+        <v>0.01266</v>
+      </c>
+      <c r="G39" s="18" t="n">
+        <v>0.00324</v>
+      </c>
+      <c r="H39" s="18" t="n">
+        <v>0.00014</v>
       </c>
     </row>
     <row r="40">
@@ -1950,49 +1950,49 @@
         </is>
       </c>
       <c r="D40" s="18" t="n">
-        <v>0.4787</v>
+        <v>0.45692</v>
       </c>
       <c r="E40" s="18" t="n">
-        <v>0.0696</v>
+        <v>0.05902</v>
       </c>
       <c r="F40" s="18" t="n">
-        <v>0.02686</v>
+        <v>0.0217</v>
       </c>
       <c r="G40" s="18" t="n">
-        <v>0.00668</v>
+        <v>0.00488</v>
       </c>
       <c r="H40" s="18" t="n">
-        <v>0.00018</v>
+        <v>0.00014</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="15" t="inlineStr">
-        <is>
-          <t>TCU</t>
-        </is>
-      </c>
-      <c r="B41" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="C41" s="15" t="inlineStr">
-        <is>
-          <t>East</t>
-        </is>
-      </c>
-      <c r="D41" s="18" t="n">
-        <v>0.39064</v>
-      </c>
-      <c r="E41" s="18" t="n">
-        <v>0.04282</v>
-      </c>
-      <c r="F41" s="18" t="n">
-        <v>0.0134</v>
-      </c>
-      <c r="G41" s="18" t="n">
-        <v>0.00344</v>
-      </c>
-      <c r="H41" s="18" t="n">
-        <v>0.00014</v>
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>Santa Clara</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="C41" s="19" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="D41" s="21" t="n">
+        <v>0.4545</v>
+      </c>
+      <c r="E41" s="21" t="n">
+        <v>0.09786</v>
+      </c>
+      <c r="F41" s="21" t="n">
+        <v>0.03028</v>
+      </c>
+      <c r="G41" s="21" t="n">
+        <v>0.0065</v>
+      </c>
+      <c r="H41" s="21" t="n">
+        <v>0.00012</v>
       </c>
     </row>
     <row r="42">
@@ -2010,19 +2010,19 @@
         </is>
       </c>
       <c r="D42" s="21" t="n">
-        <v>0.40286</v>
+        <v>0.38532</v>
       </c>
       <c r="E42" s="21" t="n">
-        <v>0.10132</v>
+        <v>0.09112000000000001</v>
       </c>
       <c r="F42" s="21" t="n">
-        <v>0.02188</v>
+        <v>0.0179</v>
       </c>
       <c r="G42" s="21" t="n">
-        <v>0.00356</v>
+        <v>0.00256</v>
       </c>
       <c r="H42" s="21" t="n">
-        <v>0.0001</v>
+        <v>8.000000000000001e-05</v>
       </c>
     </row>
     <row r="43">
@@ -2040,19 +2040,19 @@
         </is>
       </c>
       <c r="D43" s="21" t="n">
-        <v>0.35974</v>
+        <v>0.38146</v>
       </c>
       <c r="E43" s="21" t="n">
-        <v>0.06134</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.0166</v>
+        <v>0.01758</v>
       </c>
       <c r="G43" s="21" t="n">
-        <v>0.0026</v>
+        <v>0.00266</v>
       </c>
       <c r="H43" s="21" t="n">
-        <v>4e-05</v>
+        <v>8.000000000000001e-05</v>
       </c>
     </row>
     <row r="44">
@@ -2070,16 +2070,16 @@
         </is>
       </c>
       <c r="D44" s="21" t="n">
-        <v>0.39468</v>
+        <v>0.4061</v>
       </c>
       <c r="E44" s="21" t="n">
-        <v>0.06562</v>
+        <v>0.06818</v>
       </c>
       <c r="F44" s="21" t="n">
-        <v>0.01124</v>
+        <v>0.01214</v>
       </c>
       <c r="G44" s="21" t="n">
-        <v>0.00222</v>
+        <v>0.00246</v>
       </c>
       <c r="H44" s="21" t="n">
         <v>4e-05</v>
@@ -2088,11 +2088,11 @@
     <row r="45">
       <c r="A45" s="19" t="inlineStr">
         <is>
-          <t>Miami OH/SMU</t>
+          <t>Akron</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
@@ -2100,16 +2100,16 @@
         </is>
       </c>
       <c r="D45" s="21" t="n">
-        <v>0.2576</v>
+        <v>0.24818</v>
       </c>
       <c r="E45" s="21" t="n">
-        <v>0.07784000000000001</v>
+        <v>0.0558</v>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.01748</v>
+        <v>0.00534</v>
       </c>
       <c r="G45" s="21" t="n">
-        <v>0.00294</v>
+        <v>0.00078</v>
       </c>
       <c r="H45" s="21" t="n">
         <v>4e-05</v>
@@ -2118,11 +2118,11 @@
     <row r="46">
       <c r="A46" s="19" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>South Florida</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
@@ -2130,16 +2130,16 @@
         </is>
       </c>
       <c r="D46" s="21" t="n">
-        <v>0.27904</v>
+        <v>0.2393</v>
       </c>
       <c r="E46" s="21" t="n">
-        <v>0.04508</v>
+        <v>0.05364</v>
       </c>
       <c r="F46" s="21" t="n">
-        <v>0.00812</v>
+        <v>0.0125</v>
       </c>
       <c r="G46" s="21" t="n">
-        <v>0.00088</v>
+        <v>0.00202</v>
       </c>
       <c r="H46" s="21" t="n">
         <v>2e-05</v>
@@ -2148,150 +2148,150 @@
     <row r="47">
       <c r="A47" s="19" t="inlineStr">
         <is>
-          <t>Akron</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>East</t>
         </is>
       </c>
       <c r="D47" s="21" t="n">
-        <v>0.23456</v>
+        <v>0.26732</v>
       </c>
       <c r="E47" s="21" t="n">
-        <v>0.05026</v>
+        <v>0.04144</v>
       </c>
       <c r="F47" s="21" t="n">
-        <v>0.00432</v>
+        <v>0.00666</v>
       </c>
       <c r="G47" s="21" t="n">
-        <v>0.00052</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="H47" s="21" t="n">
         <v>2e-05</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="inlineStr">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
+          <t>Miami OH/SMU</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="C48" s="19" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="D48" s="21" t="n">
+        <v>0.24248</v>
+      </c>
+      <c r="E48" s="21" t="n">
+        <v>0.0667</v>
+      </c>
+      <c r="F48" s="21" t="n">
+        <v>0.01394</v>
+      </c>
+      <c r="G48" s="21" t="n">
+        <v>0.00214</v>
+      </c>
+      <c r="H48" s="21" t="n">
+        <v>2e-05</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="22" t="inlineStr">
         <is>
           <t>Siena</t>
         </is>
       </c>
-      <c r="B48" s="23" t="n">
+      <c r="B49" s="23" t="n">
         <v>16</v>
       </c>
-      <c r="C48" s="22" t="inlineStr">
+      <c r="C49" s="22" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="D48" s="24" t="n">
-        <v>0.01272</v>
-      </c>
-      <c r="E48" s="24" t="n">
-        <v>0.00086</v>
-      </c>
-      <c r="F48" s="24" t="n">
-        <v>6e-05</v>
-      </c>
-      <c r="G48" s="24" t="n">
+      <c r="D49" s="24" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="E49" s="24" t="n">
+        <v>0.00074</v>
+      </c>
+      <c r="F49" s="24" t="n">
+        <v>2e-05</v>
+      </c>
+      <c r="G49" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="24" t="n">
+      <c r="H49" s="24" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="19" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t>Northern Iowa</t>
         </is>
       </c>
-      <c r="B49" s="20" t="n">
+      <c r="B50" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="C49" s="19" t="inlineStr">
+      <c r="C50" s="19" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="D49" s="21" t="n">
-        <v>0.16422</v>
-      </c>
-      <c r="E49" s="21" t="n">
-        <v>0.0397</v>
-      </c>
-      <c r="F49" s="21" t="n">
-        <v>0.00308</v>
-      </c>
-      <c r="G49" s="21" t="n">
-        <v>0.00038</v>
-      </c>
-      <c r="H49" s="21" t="n">
+      <c r="D50" s="21" t="n">
+        <v>0.16398</v>
+      </c>
+      <c r="E50" s="21" t="n">
+        <v>0.04022</v>
+      </c>
+      <c r="F50" s="21" t="n">
+        <v>0.00316</v>
+      </c>
+      <c r="G50" s="21" t="n">
+        <v>0.00042</v>
+      </c>
+      <c r="H50" s="21" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="22" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="22" t="inlineStr">
         <is>
           <t>Cal Baptist</t>
         </is>
       </c>
-      <c r="B50" s="23" t="n">
+      <c r="B51" s="23" t="n">
         <v>13</v>
       </c>
-      <c r="C50" s="22" t="inlineStr">
+      <c r="C51" s="22" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="D50" s="24" t="n">
-        <v>0.12402</v>
-      </c>
-      <c r="E50" s="24" t="n">
-        <v>0.01516</v>
-      </c>
-      <c r="F50" s="24" t="n">
-        <v>0.00082</v>
-      </c>
-      <c r="G50" s="24" t="n">
+      <c r="D51" s="24" t="n">
+        <v>0.12046</v>
+      </c>
+      <c r="E51" s="24" t="n">
+        <v>0.01384</v>
+      </c>
+      <c r="F51" s="24" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="G51" s="24" t="n">
         <v>8.000000000000001e-05</v>
       </c>
-      <c r="H50" s="24" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="19" t="inlineStr">
-        <is>
-          <t>South Florida</t>
-        </is>
-      </c>
-      <c r="B51" s="20" t="n">
-        <v>11</v>
-      </c>
-      <c r="C51" s="19" t="inlineStr">
-        <is>
-          <t>East</t>
-        </is>
-      </c>
-      <c r="D51" s="21" t="n">
-        <v>0.23248</v>
-      </c>
-      <c r="E51" s="21" t="n">
-        <v>0.05172</v>
-      </c>
-      <c r="F51" s="21" t="n">
-        <v>0.01168</v>
-      </c>
-      <c r="G51" s="21" t="n">
-        <v>0.00178</v>
-      </c>
-      <c r="H51" s="21" t="n">
+      <c r="H51" s="24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2310,16 +2310,16 @@
         </is>
       </c>
       <c r="D52" s="24" t="n">
-        <v>0.07566000000000001</v>
+        <v>0.06691999999999999</v>
       </c>
       <c r="E52" s="24" t="n">
-        <v>0.008240000000000001</v>
+        <v>0.00624</v>
       </c>
       <c r="F52" s="24" t="n">
-        <v>0.00066</v>
+        <v>0.00046</v>
       </c>
       <c r="G52" s="24" t="n">
-        <v>4e-05</v>
+        <v>2e-05</v>
       </c>
       <c r="H52" s="24" t="n">
         <v>0</v>
@@ -2340,13 +2340,13 @@
         </is>
       </c>
       <c r="D53" s="24" t="n">
-        <v>0.03772</v>
+        <v>0.03568</v>
       </c>
       <c r="E53" s="24" t="n">
-        <v>0.00428</v>
+        <v>0.00382</v>
       </c>
       <c r="F53" s="24" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
       <c r="G53" s="24" t="n">
         <v>0</v>
@@ -2370,10 +2370,10 @@
         </is>
       </c>
       <c r="D54" s="24" t="n">
-        <v>0.00876</v>
+        <v>0.008</v>
       </c>
       <c r="E54" s="24" t="n">
-        <v>0.00056</v>
+        <v>0.00042</v>
       </c>
       <c r="F54" s="24" t="n">
         <v>4e-05</v>
@@ -2400,13 +2400,13 @@
         </is>
       </c>
       <c r="D55" s="21" t="n">
-        <v>0.1863</v>
+        <v>0.18148</v>
       </c>
       <c r="E55" s="21" t="n">
-        <v>0.03148</v>
+        <v>0.02922</v>
       </c>
       <c r="F55" s="21" t="n">
-        <v>0.00204</v>
+        <v>0.00176</v>
       </c>
       <c r="G55" s="21" t="n">
         <v>0.0002</v>
@@ -2430,16 +2430,16 @@
         </is>
       </c>
       <c r="D56" s="24" t="n">
-        <v>0.09478</v>
+        <v>0.08918</v>
       </c>
       <c r="E56" s="24" t="n">
-        <v>0.01448</v>
+        <v>0.01304</v>
       </c>
       <c r="F56" s="24" t="n">
-        <v>0.00074</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="G56" s="24" t="n">
-        <v>4e-05</v>
+        <v>2e-05</v>
       </c>
       <c r="H56" s="24" t="n">
         <v>0</v>
@@ -2460,13 +2460,13 @@
         </is>
       </c>
       <c r="D57" s="24" t="n">
-        <v>0.06673999999999999</v>
+        <v>0.06519999999999999</v>
       </c>
       <c r="E57" s="24" t="n">
-        <v>0.00894</v>
+        <v>0.0086</v>
       </c>
       <c r="F57" s="24" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.00054</v>
       </c>
       <c r="G57" s="24" t="n">
         <v>6e-05</v>
@@ -2490,10 +2490,10 @@
         </is>
       </c>
       <c r="D58" s="24" t="n">
-        <v>0.0277</v>
+        <v>0.02594</v>
       </c>
       <c r="E58" s="24" t="n">
-        <v>0.00204</v>
+        <v>0.00176</v>
       </c>
       <c r="F58" s="24" t="n">
         <v>6e-05</v>
@@ -2520,10 +2520,10 @@
         </is>
       </c>
       <c r="D59" s="24" t="n">
-        <v>0.00534</v>
+        <v>0.00476</v>
       </c>
       <c r="E59" s="24" t="n">
-        <v>0.0001</v>
+        <v>6e-05</v>
       </c>
       <c r="F59" s="24" t="n">
         <v>0</v>
@@ -2550,16 +2550,16 @@
         </is>
       </c>
       <c r="D60" s="21" t="n">
-        <v>0.18496</v>
+        <v>0.18972</v>
       </c>
       <c r="E60" s="21" t="n">
-        <v>0.04446</v>
+        <v>0.0465</v>
       </c>
       <c r="F60" s="21" t="n">
-        <v>0.00548</v>
+        <v>0.00598</v>
       </c>
       <c r="G60" s="21" t="n">
-        <v>0.00062</v>
+        <v>0.00068</v>
       </c>
       <c r="H60" s="21" t="n">
         <v>0</v>
@@ -2580,13 +2580,13 @@
         </is>
       </c>
       <c r="D61" s="24" t="n">
-        <v>0.09332</v>
+        <v>0.08734</v>
       </c>
       <c r="E61" s="24" t="n">
-        <v>0.00894</v>
+        <v>0.00742</v>
       </c>
       <c r="F61" s="24" t="n">
-        <v>0.00034</v>
+        <v>0.0002</v>
       </c>
       <c r="G61" s="24" t="n">
         <v>0</v>
@@ -2610,10 +2610,10 @@
         </is>
       </c>
       <c r="D62" s="24" t="n">
-        <v>0.04728</v>
+        <v>0.04476</v>
       </c>
       <c r="E62" s="24" t="n">
-        <v>0.00572</v>
+        <v>0.00496</v>
       </c>
       <c r="F62" s="24" t="n">
         <v>0.00026</v>
@@ -2640,13 +2640,13 @@
         </is>
       </c>
       <c r="D63" s="24" t="n">
-        <v>0.03164</v>
+        <v>0.02888</v>
       </c>
       <c r="E63" s="24" t="n">
-        <v>0.00304</v>
+        <v>0.0026</v>
       </c>
       <c r="F63" s="24" t="n">
-        <v>0.00014</v>
+        <v>8.000000000000001e-05</v>
       </c>
       <c r="G63" s="24" t="n">
         <v>0</v>
@@ -2670,10 +2670,10 @@
         </is>
       </c>
       <c r="D64" s="24" t="n">
-        <v>0.00784</v>
+        <v>0.00704</v>
       </c>
       <c r="E64" s="24" t="n">
-        <v>0.00046</v>
+        <v>0.00042</v>
       </c>
       <c r="F64" s="24" t="n">
         <v>4e-05</v>
@@ -2700,16 +2700,16 @@
         </is>
       </c>
       <c r="D65" s="24" t="n">
-        <v>0.12474</v>
+        <v>0.12644</v>
       </c>
       <c r="E65" s="24" t="n">
-        <v>0.02658</v>
+        <v>0.02784</v>
       </c>
       <c r="F65" s="24" t="n">
-        <v>0.00144</v>
+        <v>0.00148</v>
       </c>
       <c r="G65" s="24" t="n">
-        <v>0.00012</v>
+        <v>0.00014</v>
       </c>
       <c r="H65" s="24" t="n">
         <v>0</v>
@@ -2730,16 +2730,16 @@
         </is>
       </c>
       <c r="D66" s="24" t="n">
-        <v>0.07868</v>
+        <v>0.07504</v>
       </c>
       <c r="E66" s="24" t="n">
-        <v>0.00702</v>
+        <v>0.00656</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>0.00046</v>
+        <v>0.00036</v>
       </c>
       <c r="G66" s="24" t="n">
-        <v>2e-05</v>
+        <v>0</v>
       </c>
       <c r="H66" s="24" t="n">
         <v>0</v>
@@ -2760,13 +2760,13 @@
         </is>
       </c>
       <c r="D67" s="24" t="n">
-        <v>0.0281</v>
+        <v>0.02644</v>
       </c>
       <c r="E67" s="24" t="n">
-        <v>0.00198</v>
+        <v>0.0018</v>
       </c>
       <c r="F67" s="24" t="n">
-        <v>6e-05</v>
+        <v>2e-05</v>
       </c>
       <c r="G67" s="24" t="n">
         <v>0</v>
@@ -4377,7 +4377,7 @@
     <row r="2">
       <c r="A2" s="43" t="inlineStr">
         <is>
-          <t>CHAMPION: (3) Illinois  |  Upsets: 15</t>
+          <t>CHAMPION: (3) Illinois  |  Upsets: 16</t>
         </is>
       </c>
     </row>
@@ -4786,19 +4786,24 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="48" t="inlineStr">
+      <c r="A35" s="49" t="inlineStr">
         <is>
           <t>(8) Villanova</t>
         </is>
       </c>
-      <c r="B35" s="49" t="inlineStr">
+      <c r="B35" s="48" t="inlineStr">
         <is>
           <t>(9) Utah State</t>
         </is>
       </c>
-      <c r="C35" s="48" t="inlineStr">
-        <is>
-          <t>(8) Villanova</t>
+      <c r="C35" s="54" t="inlineStr">
+        <is>
+          <t>(9) Utah State</t>
+        </is>
+      </c>
+      <c r="D35" s="55" t="inlineStr">
+        <is>
+          <t>UPSET</t>
         </is>
       </c>
     </row>
@@ -4946,7 +4951,7 @@
       </c>
       <c r="B45" s="49" t="inlineStr">
         <is>
-          <t>(8) Villanova</t>
+          <t>(9) Utah State</t>
         </is>
       </c>
       <c r="C45" s="46" t="inlineStr">
@@ -9086,7 +9091,7 @@
     <row r="2">
       <c r="A2" s="43" t="inlineStr">
         <is>
-          <t>CHAMPION: (3) Gonzaga  |  Upsets: 19</t>
+          <t>CHAMPION: (3) Gonzaga  |  Upsets: 20</t>
         </is>
       </c>
     </row>
@@ -10244,19 +10249,24 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="50" t="inlineStr">
+      <c r="A90" s="53" t="inlineStr">
         <is>
           <t>(5) Texas Tech</t>
         </is>
       </c>
-      <c r="B90" s="51" t="inlineStr">
+      <c r="B90" s="65" t="inlineStr">
         <is>
           <t>(12) Akron</t>
         </is>
       </c>
-      <c r="C90" s="50" t="inlineStr">
-        <is>
-          <t>(5) Texas Tech</t>
+      <c r="C90" s="54" t="inlineStr">
+        <is>
+          <t>(12) Akron</t>
+        </is>
+      </c>
+      <c r="D90" s="55" t="inlineStr">
+        <is>
+          <t>UPSET</t>
         </is>
       </c>
     </row>
@@ -10402,9 +10412,9 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="50" t="inlineStr">
-        <is>
-          <t>(5) Texas Tech</t>
+      <c r="A100" s="65" t="inlineStr">
+        <is>
+          <t>(12) Akron</t>
         </is>
       </c>
       <c r="B100" s="47" t="inlineStr">
@@ -10412,9 +10422,9 @@
           <t>(13) Hofstra</t>
         </is>
       </c>
-      <c r="C100" s="50" t="inlineStr">
-        <is>
-          <t>(5) Texas Tech</t>
+      <c r="C100" s="65" t="inlineStr">
+        <is>
+          <t>(12) Akron</t>
         </is>
       </c>
     </row>
@@ -10492,9 +10502,9 @@
           <t>(1) Michigan</t>
         </is>
       </c>
-      <c r="B106" s="53" t="inlineStr">
-        <is>
-          <t>(5) Texas Tech</t>
+      <c r="B106" s="51" t="inlineStr">
+        <is>
+          <t>(12) Akron</t>
         </is>
       </c>
       <c r="C106" s="46" t="inlineStr">
@@ -10684,7 +10694,7 @@
     <row r="2">
       <c r="A2" s="43" t="inlineStr">
         <is>
-          <t>CHAMPION: (1) Arizona  |  Upsets: 15</t>
+          <t>CHAMPION: (1) Arizona  |  Upsets: 16</t>
         </is>
       </c>
     </row>
@@ -11476,19 +11486,24 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="50" t="inlineStr">
+      <c r="A63" s="53" t="inlineStr">
         <is>
           <t>(5) Vanderbilt</t>
         </is>
       </c>
-      <c r="B63" s="51" t="inlineStr">
+      <c r="B63" s="65" t="inlineStr">
         <is>
           <t>(12) McNeese</t>
         </is>
       </c>
-      <c r="C63" s="50" t="inlineStr">
-        <is>
-          <t>(5) Vanderbilt</t>
+      <c r="C63" s="54" t="inlineStr">
+        <is>
+          <t>(12) McNeese</t>
+        </is>
+      </c>
+      <c r="D63" s="55" t="inlineStr">
+        <is>
+          <t>UPSET</t>
         </is>
       </c>
     </row>
@@ -11629,9 +11644,9 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="53" t="inlineStr">
-        <is>
-          <t>(5) Vanderbilt</t>
+      <c r="A73" s="51" t="inlineStr">
+        <is>
+          <t>(12) McNeese</t>
         </is>
       </c>
       <c r="B73" s="50" t="inlineStr">
@@ -12257,7 +12272,7 @@
     <row r="2">
       <c r="A2" s="43" t="inlineStr">
         <is>
-          <t>CHAMPION: (1) Florida  |  Upsets: 14</t>
+          <t>CHAMPION: (1) Florida  |  Upsets: 13</t>
         </is>
       </c>
     </row>
@@ -12943,24 +12958,19 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="65" t="inlineStr">
+      <c r="A53" s="51" t="inlineStr">
         <is>
           <t>(11) Texas/NC State</t>
         </is>
       </c>
-      <c r="B53" s="56" t="inlineStr">
+      <c r="B53" s="52" t="inlineStr">
         <is>
           <t>(2) Purdue</t>
         </is>
       </c>
-      <c r="C53" s="54" t="inlineStr">
-        <is>
-          <t>(11) Texas/NC State</t>
-        </is>
-      </c>
-      <c r="D53" s="55" t="inlineStr">
-        <is>
-          <t>UPSET</t>
+      <c r="C53" s="52" t="inlineStr">
+        <is>
+          <t>(2) Purdue</t>
         </is>
       </c>
     </row>
@@ -12977,9 +12987,9 @@
           <t>(1) Arizona</t>
         </is>
       </c>
-      <c r="B56" s="70" t="inlineStr">
-        <is>
-          <t>(11) Texas/NC State</t>
+      <c r="B56" s="58" t="inlineStr">
+        <is>
+          <t>(2) Purdue</t>
         </is>
       </c>
       <c r="C56" s="57" t="inlineStr">
@@ -15393,7 +15403,7 @@
     <row r="2">
       <c r="A2" s="43" t="inlineStr">
         <is>
-          <t>CHAMPION: (1) Florida  |  Upsets: 14</t>
+          <t>CHAMPION: (1) Florida  |  Upsets: 13</t>
         </is>
       </c>
     </row>
@@ -16103,24 +16113,19 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="66" t="inlineStr">
+      <c r="A56" s="68" t="inlineStr">
         <is>
           <t>(4) Arkansas</t>
         </is>
       </c>
-      <c r="B56" s="73" t="inlineStr">
+      <c r="B56" s="74" t="inlineStr">
         <is>
           <t>(7) Miami FL</t>
         </is>
       </c>
-      <c r="C56" s="73" t="inlineStr">
-        <is>
-          <t>(7) Miami FL — West CHAMP</t>
-        </is>
-      </c>
-      <c r="D56" s="55" t="inlineStr">
-        <is>
-          <t>UPSET</t>
+      <c r="C56" s="68" t="inlineStr">
+        <is>
+          <t>(4) Arkansas — West CHAMP</t>
         </is>
       </c>
     </row>
@@ -16863,7 +16868,7 @@
       </c>
       <c r="B114" s="59" t="inlineStr">
         <is>
-          <t>(7) Miami FL [West]</t>
+          <t>(4) Arkansas [West]</t>
         </is>
       </c>
       <c r="C114" s="57" t="inlineStr">
@@ -18596,7 +18601,7 @@
         <v>4</v>
       </c>
       <c r="E4" s="27" t="n">
-        <v>0.09528</v>
+        <v>0.09637999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -18617,7 +18622,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="27" t="n">
-        <v>0.20802</v>
+        <v>0.21246</v>
       </c>
     </row>
     <row r="6">
@@ -18638,7 +18643,7 @@
         <v>3</v>
       </c>
       <c r="E6" s="27" t="n">
-        <v>0.14568</v>
+        <v>0.14904</v>
       </c>
     </row>
     <row r="7">
@@ -18659,7 +18664,7 @@
         <v>2</v>
       </c>
       <c r="E7" s="27" t="n">
-        <v>0.05528</v>
+        <v>0.0547</v>
       </c>
     </row>
     <row r="8">
@@ -18680,7 +18685,7 @@
         <v>2</v>
       </c>
       <c r="E8" s="27" t="n">
-        <v>0.01842</v>
+        <v>0.01694</v>
       </c>
     </row>
     <row r="9">
@@ -18701,7 +18706,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="27" t="n">
-        <v>0.15586</v>
+        <v>0.15978</v>
       </c>
     </row>
     <row r="10">
@@ -18722,7 +18727,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="27" t="n">
-        <v>0.07876</v>
+        <v>0.07716000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -18743,7 +18748,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="27" t="n">
-        <v>0.0098</v>
+        <v>0.01004</v>
       </c>
     </row>
     <row r="12">
@@ -18764,7 +18769,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="27" t="n">
-        <v>0.05154</v>
+        <v>0.05102</v>
       </c>
     </row>
     <row r="13">
@@ -18785,7 +18790,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="27" t="n">
-        <v>0.02944</v>
+        <v>0.02416</v>
       </c>
     </row>
     <row r="14">
@@ -18806,7 +18811,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="27" t="n">
-        <v>0.00224</v>
+        <v>0.00176</v>
       </c>
     </row>
   </sheetData>
@@ -19813,24 +19818,19 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="51" t="inlineStr">
+      <c r="A73" s="65" t="inlineStr">
         <is>
           <t>(12) McNeese</t>
         </is>
       </c>
-      <c r="B73" s="69" t="inlineStr">
+      <c r="B73" s="47" t="inlineStr">
         <is>
           <t>(13) Troy</t>
         </is>
       </c>
-      <c r="C73" s="54" t="inlineStr">
-        <is>
-          <t>(13) Troy</t>
-        </is>
-      </c>
-      <c r="D73" s="55" t="inlineStr">
-        <is>
-          <t>UPSET</t>
+      <c r="C73" s="65" t="inlineStr">
+        <is>
+          <t>(12) McNeese</t>
         </is>
       </c>
     </row>
@@ -19908,9 +19908,9 @@
           <t>(1) Florida</t>
         </is>
       </c>
-      <c r="B79" s="47" t="inlineStr">
-        <is>
-          <t>(13) Troy</t>
+      <c r="B79" s="51" t="inlineStr">
+        <is>
+          <t>(12) McNeese</t>
         </is>
       </c>
       <c r="C79" s="46" t="inlineStr">
@@ -20259,19 +20259,24 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="46" t="inlineStr">
+      <c r="A106" s="67" t="inlineStr">
         <is>
           <t>(1) Michigan</t>
         </is>
       </c>
-      <c r="B106" s="51" t="inlineStr">
+      <c r="B106" s="65" t="inlineStr">
         <is>
           <t>(12) Akron</t>
         </is>
       </c>
-      <c r="C106" s="46" t="inlineStr">
-        <is>
-          <t>(1) Michigan</t>
+      <c r="C106" s="54" t="inlineStr">
+        <is>
+          <t>(12) Akron</t>
+        </is>
+      </c>
+      <c r="D106" s="55" t="inlineStr">
+        <is>
+          <t>UPSET</t>
         </is>
       </c>
     </row>
@@ -20305,19 +20310,19 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="57" t="inlineStr">
-        <is>
-          <t>(1) Michigan</t>
-        </is>
-      </c>
-      <c r="B110" s="66" t="inlineStr">
+      <c r="A110" s="70" t="inlineStr">
+        <is>
+          <t>(12) Akron</t>
+        </is>
+      </c>
+      <c r="B110" s="68" t="inlineStr">
         <is>
           <t>(6) Tennessee</t>
         </is>
       </c>
-      <c r="C110" s="57" t="inlineStr">
-        <is>
-          <t>(1) Michigan — Midwest CHAMP</t>
+      <c r="C110" s="68" t="inlineStr">
+        <is>
+          <t>(6) Tennessee — Midwest CHAMP</t>
         </is>
       </c>
     </row>
@@ -20348,7 +20353,7 @@
     <row r="114">
       <c r="A114" s="59" t="inlineStr">
         <is>
-          <t>(1) Michigan [Midwest]</t>
+          <t>(6) Tennessee [Midwest]</t>
         </is>
       </c>
       <c r="B114" s="60" t="inlineStr">
@@ -20359,11 +20364,6 @@
       <c r="C114" s="72" t="inlineStr">
         <is>
           <t>(3) Gonzaga</t>
-        </is>
-      </c>
-      <c r="D114" s="55" t="inlineStr">
-        <is>
-          <t>UPSET</t>
         </is>
       </c>
     </row>
@@ -27335,9 +27335,9 @@
           <t>Utah State</t>
         </is>
       </c>
-      <c r="K21" s="77" t="inlineStr">
-        <is>
-          <t>Villanova</t>
+      <c r="K21" s="78" t="inlineStr">
+        <is>
+          <t>Utah State</t>
         </is>
       </c>
       <c r="L21" s="77" t="inlineStr">
@@ -28764,9 +28764,9 @@
           <t>(3) Gonzaga</t>
         </is>
       </c>
-      <c r="P33" s="84" t="inlineStr">
-        <is>
-          <t>(11) Texas/NC State</t>
+      <c r="P33" s="83" t="inlineStr">
+        <is>
+          <t>(2) Purdue</t>
         </is>
       </c>
       <c r="Q33" s="83" t="inlineStr">
@@ -28891,9 +28891,9 @@
           <t>(1) Arizona</t>
         </is>
       </c>
-      <c r="R34" s="88" t="inlineStr">
-        <is>
-          <t>(7) Miami FL</t>
+      <c r="R34" s="86" t="inlineStr">
+        <is>
+          <t>(4) Arkansas</t>
         </is>
       </c>
       <c r="S34" s="85" t="inlineStr">
@@ -29227,9 +29227,9 @@
           <t>Vanderbilt</t>
         </is>
       </c>
-      <c r="O38" s="77" t="inlineStr">
-        <is>
-          <t>Vanderbilt</t>
+      <c r="O38" s="78" t="inlineStr">
+        <is>
+          <t>McNeese</t>
         </is>
       </c>
       <c r="P38" s="77" t="inlineStr">
@@ -30073,7 +30073,7 @@
       </c>
       <c r="T45" s="79" t="inlineStr">
         <is>
-          <t>(13) Troy</t>
+          <t>(12) McNeese</t>
         </is>
       </c>
       <c r="U45" s="79" t="inlineStr">
@@ -30977,9 +30977,9 @@
           <t>Texas Tech</t>
         </is>
       </c>
-      <c r="N54" s="77" t="inlineStr">
-        <is>
-          <t>Texas Tech</t>
+      <c r="N54" s="78" t="inlineStr">
+        <is>
+          <t>Akron</t>
         </is>
       </c>
       <c r="O54" s="77" t="inlineStr">
@@ -31798,7 +31798,7 @@
       </c>
       <c r="N61" s="79" t="inlineStr">
         <is>
-          <t>(5) Texas Tech</t>
+          <t>(12) Akron</t>
         </is>
       </c>
       <c r="O61" s="79" t="inlineStr">
@@ -32177,9 +32177,9 @@
           <t>(9) Saint Louis</t>
         </is>
       </c>
-      <c r="T64" s="80" t="inlineStr">
-        <is>
-          <t>(1) Michigan</t>
+      <c r="T64" s="84" t="inlineStr">
+        <is>
+          <t>(12) Akron</t>
         </is>
       </c>
       <c r="U64" s="82" t="inlineStr">
@@ -32411,9 +32411,9 @@
           <t>(2) Iowa State</t>
         </is>
       </c>
-      <c r="T66" s="85" t="inlineStr">
-        <is>
-          <t>(1) Michigan</t>
+      <c r="T66" s="86" t="inlineStr">
+        <is>
+          <t>(6) Tennessee</t>
         </is>
       </c>
       <c r="U66" s="87" t="inlineStr">

</xml_diff>